<commit_message>
docs(flight): record the final pre-search suggestion rules
The suggestions reference now says a departure-only turn gets no search, fare or cheapest-destination suggestion. The register cites c02b4d9 for G19 and for Step 6, and its Evidence sheet is re-tallied from the final live runs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/flight-suggested-questions-gap-analysis.xlsx
+++ b/docs/flight-suggested-questions-gap-analysis.xlsx
@@ -1349,7 +1349,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed in 3915f3b and 047f9cd</t>
+          <t xml:space="preserve">Fixed in 3915f3b, 047f9cd and c02b4d9</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1777,7 +1777,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generated: 2026-10-01T14:21:43.876Z</t>
+          <t xml:space="preserve">Generated: 2026-10-01T14:29:46.108Z</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4221,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done in 3915f3b, 5625dd8, 047f9cd and a340ee2; G21 and G22 only partly, by design</t>
+          <t xml:space="preserve">Done in 3915f3b, 5625dd8, 047f9cd, a340ee2 and c02b4d9; G21 and G22 only partly, by design</t>
         </is>
       </c>
     </row>

</xml_diff>